<commit_message>
enabling gtithub pipeline and updated  instructions
</commit_message>
<xml_diff>
--- a/docs/Test_Plan_and_Test_Cases.xlsx
+++ b/docs/Test_Plan_and_Test_Cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rjdgo\Documents\Workspace\selenium\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B14FDDF-2AAE-49A9-9805-CBED6B81BC4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1F8A30A-A177-4A90-9F1F-D20B684DC8B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="29580" yWindow="780" windowWidth="38700" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -234,7 +234,7 @@
     <t>API rate limiting</t>
   </si>
   <si>
-    <t>reqres.in returns rate-limit headers (20 requests per 60 seconds observed). Mitigation: keep the API suite small and avoid parallel API runs.</t>
+    <t>reqres.in allows 40 requests per day per IP address without an account (plus a 20 requests/minute window). When the limit is used up, API cases fail with 429 'rate_limit_exceeded' until midnight UTC. Mitigation: avoid repeated API runs, run API tests once per cycle with -Dcucumber.filter.tags=@API, or use a reqres.in account for a higher limit.</t>
   </si>
   <si>
     <t>Browser / driver drift</t>
@@ -276,7 +276,7 @@
   <si>
     <t>mvn clean test -Denv=qa
 Optional: -Dbrowser=firefox -Dheadless=true
-The runner executes everything tagged @All; to run a subset, change the tag filter in TestRunner.java.</t>
+Run a subset by tag: "-Dcucumber.filter.tags=@API" (default @All; keep the quotes in PowerShell).</t>
   </si>
   <si>
     <t>13. Roles and responsibilities</t>
@@ -3990,7 +3990,7 @@
       </c>
       <c r="R19" s="4"/>
     </row>
-    <row r="20" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:18" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>291</v>
       </c>

</xml_diff>